<commit_message>
resolved the issue of mapping
</commit_message>
<xml_diff>
--- a/mapping.xlsx
+++ b/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Export Summary" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="126">
   <si>
     <t xml:space="preserve">This document was exported from Numbers. Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -373,6 +373,9 @@
   </si>
   <si>
     <t xml:space="preserve">ReferenceColumn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LookupField</t>
   </si>
   <si>
     <t xml:space="preserve">departments</t>
@@ -407,7 +410,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -456,11 +459,6 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -476,7 +474,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -512,13 +510,6 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -545,7 +536,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -595,14 +586,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2832,7 +2815,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="5" width="20.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="5" width="37.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="5" width="20.83"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="5" style="5" width="8.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="5" width="19.51"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="6" style="5" width="8.85"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2848,11 +2832,13 @@
       <c r="D1" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="E1" s="9"/>
+      <c r="E1" s="9" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>16</v>
@@ -2861,13 +2847,15 @@
         <v>100</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E2" s="9"/>
+        <v>119</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>16</v>
@@ -2876,13 +2864,15 @@
         <v>102</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E3" s="9"/>
+        <v>119</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>16</v>
@@ -2891,13 +2881,15 @@
         <v>93</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E4" s="9"/>
+        <v>119</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>16</v>
@@ -2906,13 +2898,15 @@
         <v>104</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E5" s="9"/>
+        <v>119</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>16</v>
@@ -2921,12 +2915,14 @@
         <v>87</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E6" s="9"/>
+        <v>119</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="7" t="s">
         <v>96</v>
       </c>
       <c r="B7" s="7" t="s">
@@ -2936,12 +2932,14 @@
         <v>28</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E7" s="9"/>
+        <v>119</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="7" t="s">
         <v>96</v>
       </c>
       <c r="B8" s="7" t="s">
@@ -2951,13 +2949,15 @@
         <v>24</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E8" s="9"/>
+        <v>119</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>16</v>
@@ -2966,13 +2966,15 @@
         <v>20</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E9" s="9"/>
+        <v>119</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>16</v>
@@ -2981,13 +2983,15 @@
         <v>45</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E10" s="14"/>
+        <v>119</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>16</v>
@@ -2996,12 +3000,15 @@
         <v>32</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>16</v>
@@ -3010,12 +3017,15 @@
         <v>77</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>16</v>
@@ -3024,7 +3034,10 @@
         <v>81</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
handled all json data in db that are refered
</commit_message>
<xml_diff>
--- a/mapping.xlsx
+++ b/mapping.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="128">
   <si>
     <t xml:space="preserve">This document was exported from Numbers. Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -396,10 +396,16 @@
     <t xml:space="preserve">organizations</t>
   </si>
   <si>
+    <t xml:space="preserve">value-&gt;&gt;'name'</t>
+  </si>
+  <si>
     <t xml:space="preserve">status_master</t>
   </si>
   <si>
     <t xml:space="preserve">users</t>
+  </si>
+  <si>
+    <t xml:space="preserve">first_name</t>
   </si>
 </sst>
 </file>
@@ -410,7 +416,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -458,6 +464,11 @@
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="3">
@@ -536,7 +547,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -587,6 +598,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2931,11 +2946,11 @@
       <c r="C7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="13" t="s">
         <v>119</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>15</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2948,16 +2963,16 @@
       <c r="C8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="13" t="s">
         <v>119</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>15</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>16</v>
@@ -2974,7 +2989,7 @@
     </row>
     <row r="10" customFormat="false" ht="13.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>16</v>
@@ -2991,7 +3006,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>16</v>
@@ -3008,7 +3023,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>16</v>
@@ -3020,12 +3035,12 @@
         <v>119</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>15</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>16</v>

</xml_diff>